<commit_message>
Fix Phase-1 vacant count (81) and add Plan281 Deployed/Selected/Pending
Cross-check Summary172: Transport vacant corrected 7→6 so total vacant is 81 (172−91), not 82. Analysis sheet 4 now shows Required/Filled/Vacant (all ≥0). DesignationSummary negatives replaced with Shortfall/Surplus. Plan281 gains Deployed, Selected, Pending columns from DailySheet status.

Co-authored-by: Srikar Bokka <Srikar6266@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Phase1_172_vs_281_Manpower_Analysis_Report.xlsx
+++ b/Phase1_172_vs_281_Manpower_Analysis_Report.xlsx
@@ -113,7 +113,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -135,11 +135,104 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -218,6 +311,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -772,6 +877,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1001,6 +1107,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -1014,9 +1121,27 @@
           <t>Phase-1 needs 172 people immediately against a full plan of 281 (109 deferred). Against the full 281 plan we currently have 159 people in the manpower list (141 deployed + 18 will join), leaving a 122-person gap to full plan. Against the Phase-1 172 roster, 91 slots are named (53%) and 81 slots remain vacant (47%). Biggest Phase-1 risks: ELV/SCADA is 0/10 filled; Admin leadership still missing Sr Managers / HSE / Materials; Mechanical has the largest vacant block. Against full 281, largest hiring gaps are Runway Team (−13), HVAC Technicians (−10), Civil Helpers (−8), Pump Operators (−8), and Electrical Shift Engineers (−7).</t>
         </is>
       </c>
-    </row>
-    <row r="19"/>
-    <row r="20"/>
+      <c r="B18" s="34" t="n"/>
+      <c r="C18" s="34" t="n"/>
+      <c r="D18" s="34" t="n"/>
+      <c r="E18" s="34" t="n"/>
+      <c r="F18" s="34" t="n"/>
+      <c r="G18" s="35" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="36" t="n"/>
+      <c r="G19" s="37" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="38" t="n"/>
+      <c r="B20" s="39" t="n"/>
+      <c r="C20" s="39" t="n"/>
+      <c r="D20" s="39" t="n"/>
+      <c r="E20" s="39" t="n"/>
+      <c r="F20" s="39" t="n"/>
+      <c r="G20" s="40" t="n"/>
+    </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
@@ -1238,6 +1363,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
@@ -1428,7 +1554,7 @@
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>82%</t>
+          <t>81%</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
@@ -1622,7 +1748,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Difference (Deferred)</t>
+          <t>Difference (absolute / positive)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -1665,11 +1791,11 @@
         <v>8</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>Ph-1 ELV scope (10) vs Plan B SCADA+Helpdesk (8) — naming differs; ELV floor techs are Ph-1 specific</t>
+          <t>Ph-1 ELV scope (10) vs Plan B SCADA+Helpdesk (8) — naming differs; ELV floor techs are Ph-1 specific | Shown as positive Ph-1 excess vs 281 grouping.</t>
         </is>
       </c>
     </row>
@@ -1686,11 +1812,11 @@
         <v>56</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>-33</v>
+        <v>33</v>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>Ph-1 Mechanical 89 includes plumbing/pump/sewer/WTP items that sit under Civil (F) in 281 plan</t>
+          <t>Ph-1 Mechanical 89 includes plumbing/pump/sewer/WTP items that sit under Civil (F) in 281 plan | Shown as positive Ph-1 excess vs 281 grouping.</t>
         </is>
       </c>
     </row>
@@ -1820,6 +1946,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -1836,6 +1963,7 @@
     </row>
     <row r="18"/>
     <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -1890,7 +2018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1898,8 +2026,9 @@
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1944,10 +2073,15 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Gap (Req−Filled)</t>
+          <t>Shortfall</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Surplus</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1976,7 +2110,10 @@
       <c r="F5" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="G5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="24" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2002,10 +2139,13 @@
       <c r="E6" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="G6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="24" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2034,7 +2174,10 @@
       <c r="F7" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="24" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2063,7 +2206,10 @@
       <c r="F8" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="24" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2092,7 +2238,10 @@
       <c r="F9" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="G9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="24" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2121,7 +2270,10 @@
       <c r="F10" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="G10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="24" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2147,10 +2299,13 @@
       <c r="E11" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="F11" s="7" t="n">
+      <c r="F11" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="24" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2176,10 +2331,13 @@
       <c r="E12" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="10" t="n">
+      <c r="F12" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2205,10 +2363,13 @@
       <c r="E13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="10" t="n">
+      <c r="F13" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2234,10 +2395,13 @@
       <c r="E14" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="10" t="n">
+      <c r="F14" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2263,10 +2427,13 @@
       <c r="E15" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="10" t="n">
+      <c r="F15" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2292,10 +2459,13 @@
       <c r="E16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="10" t="n">
+      <c r="F16" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2321,10 +2491,13 @@
       <c r="E17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="10" t="n">
+      <c r="F17" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2350,10 +2523,13 @@
       <c r="E18" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="10" t="n">
+      <c r="F18" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G18" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2379,10 +2555,13 @@
       <c r="E19" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F19" s="10" t="n">
+      <c r="F19" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2408,10 +2587,13 @@
       <c r="E20" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="10" t="n">
+      <c r="F20" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G20" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2437,10 +2619,13 @@
       <c r="E21" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="F21" s="11" t="n">
+      <c r="F21" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G21" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2466,10 +2651,13 @@
       <c r="E22" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="F22" s="11" t="n">
+      <c r="F22" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2495,10 +2683,13 @@
       <c r="E23" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F23" s="10" t="n">
+      <c r="F23" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G23" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2524,10 +2715,13 @@
       <c r="E24" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F24" s="10" t="n">
+      <c r="F24" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G24" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2553,10 +2747,13 @@
       <c r="E25" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F25" s="10" t="n">
+      <c r="F25" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G25" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2585,7 +2782,10 @@
       <c r="F26" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G26" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2611,10 +2811,13 @@
       <c r="E27" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="F27" s="11" t="n">
+      <c r="F27" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G27" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2640,10 +2843,13 @@
       <c r="E28" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F28" s="10" t="n">
+      <c r="F28" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G28" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2669,10 +2875,13 @@
       <c r="E29" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F29" s="10" t="n">
+      <c r="F29" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="G29" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2698,10 +2907,13 @@
       <c r="E30" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F30" s="10" t="n">
+      <c r="F30" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G30" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2727,10 +2939,13 @@
       <c r="E31" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F31" s="10" t="n">
+      <c r="F31" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="G31" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2756,10 +2971,13 @@
       <c r="E32" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F32" s="10" t="n">
+      <c r="F32" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G32" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2785,10 +3003,13 @@
       <c r="E33" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F33" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="F33" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2814,10 +3035,13 @@
       <c r="E34" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F34" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="F34" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2843,10 +3067,13 @@
       <c r="E35" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F35" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
+      <c r="F35" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2872,10 +3099,13 @@
       <c r="E36" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F36" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="F36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2901,10 +3131,13 @@
       <c r="E37" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F37" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="F37" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2930,10 +3163,13 @@
       <c r="E38" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F38" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="F38" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2959,10 +3195,13 @@
       <c r="E39" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F39" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" s="7" t="inlineStr">
+      <c r="F39" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -2988,10 +3227,13 @@
       <c r="E40" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F40" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G40" s="7" t="inlineStr">
+      <c r="F40" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -3020,7 +3262,10 @@
       <c r="F41" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G41" s="7" t="inlineStr">
+      <c r="G41" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -3049,7 +3294,10 @@
       <c r="F42" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G42" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -3078,7 +3326,10 @@
       <c r="F43" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G43" s="7" t="inlineStr">
+      <c r="G43" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -3104,10 +3355,13 @@
       <c r="E44" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F44" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
+      <c r="F44" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -3133,10 +3387,13 @@
       <c r="E45" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F45" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="F45" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -3162,10 +3419,13 @@
       <c r="E46" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F46" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="F46" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -3194,7 +3454,10 @@
       <c r="F47" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G47" s="7" t="inlineStr">
+      <c r="G47" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -3220,10 +3483,13 @@
       <c r="E48" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="F48" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="F48" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -3249,10 +3515,13 @@
       <c r="E49" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F49" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="F49" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -3278,10 +3547,13 @@
       <c r="E50" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F50" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="F50" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -3307,10 +3579,13 @@
       <c r="E51" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="F51" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="F51" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="22" t="inlineStr">
         <is>
           <t>SHORTFALL</t>
         </is>
@@ -3339,7 +3614,10 @@
       <c r="F52" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G52" s="8" t="inlineStr">
+      <c r="G52" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="23" t="inlineStr">
         <is>
           <t>MATCHED</t>
         </is>
@@ -3368,7 +3646,10 @@
       <c r="F53" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G53" s="8" t="inlineStr">
+      <c r="G53" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="23" t="inlineStr">
         <is>
           <t>MATCHED</t>
         </is>
@@ -3397,7 +3678,10 @@
       <c r="F54" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G54" s="8" t="inlineStr">
+      <c r="G54" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="23" t="inlineStr">
         <is>
           <t>MATCHED</t>
         </is>
@@ -3426,7 +3710,10 @@
       <c r="F55" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G55" s="8" t="inlineStr">
+      <c r="G55" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="23" t="inlineStr">
         <is>
           <t>MATCHED</t>
         </is>
@@ -3455,7 +3742,10 @@
       <c r="F56" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G56" s="8" t="inlineStr">
+      <c r="G56" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="23" t="inlineStr">
         <is>
           <t>MATCHED</t>
         </is>
@@ -3484,7 +3774,10 @@
       <c r="F57" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G57" s="8" t="inlineStr">
+      <c r="G57" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="23" t="inlineStr">
         <is>
           <t>MATCHED</t>
         </is>
@@ -3513,7 +3806,10 @@
       <c r="F58" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G58" s="8" t="inlineStr">
+      <c r="G58" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="23" t="inlineStr">
         <is>
           <t>MATCHED</t>
         </is>
@@ -3542,7 +3838,10 @@
       <c r="F59" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G59" s="8" t="inlineStr">
+      <c r="G59" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="23" t="inlineStr">
         <is>
           <t>MATCHED</t>
         </is>
@@ -3571,7 +3870,10 @@
       <c r="F60" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G60" s="8" t="inlineStr">
+      <c r="G60" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="23" t="inlineStr">
         <is>
           <t>MATCHED</t>
         </is>
@@ -3600,7 +3902,10 @@
       <c r="F61" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G61" s="8" t="inlineStr">
+      <c r="G61" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="23" t="inlineStr">
         <is>
           <t>MATCHED</t>
         </is>
@@ -3629,7 +3934,10 @@
       <c r="F62" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G62" s="8" t="inlineStr">
+      <c r="G62" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="23" t="inlineStr">
         <is>
           <t>MATCHED</t>
         </is>
@@ -3658,9 +3966,12 @@
         <v>1</v>
       </c>
       <c r="F63" s="8" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G63" s="20" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="G63" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" s="32" t="inlineStr">
         <is>
           <t>SURPLUS</t>
         </is>
@@ -3689,9 +4000,12 @@
         <v>3</v>
       </c>
       <c r="F64" s="8" t="n">
-        <v>-3</v>
-      </c>
-      <c r="G64" s="20" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="G64" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H64" s="32" t="inlineStr">
         <is>
           <t>SURPLUS</t>
         </is>
@@ -3720,9 +4034,12 @@
         <v>3</v>
       </c>
       <c r="F65" s="8" t="n">
-        <v>-3</v>
-      </c>
-      <c r="G65" s="20" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="G65" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H65" s="32" t="inlineStr">
         <is>
           <t>SURPLUS</t>
         </is>
@@ -3735,7 +4052,7 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C66" s="16" t="n"/>
+      <c r="C66" s="15" t="n"/>
       <c r="D66" s="15" t="n">
         <v>281</v>
       </c>
@@ -3743,9 +4060,16 @@
         <v>159</v>
       </c>
       <c r="F66" s="15" t="n">
-        <v>122</v>
-      </c>
-      <c r="G66" s="16" t="n"/>
+        <v>129</v>
+      </c>
+      <c r="G66" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="H66" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:G65"/>
@@ -3762,486 +4086,442 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PHASE-1 172 ROSTER — VACANT POSITIONS (HIRING LIST)</t>
+          <t>PHASE-1 172 ROSTER — REQUIRED / FILLED / VACANT (CROSS-CHECKED)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Source: Deployment172 sheet — positions where Name is empty. These are the immediate Phase-1 open slots.</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cross-check: Source Summary172 showed Vacant=82 because TRANSPORT vacant was typed as 7 (must be 10−4=6). Correct from Deployment172: Required 172 | Filled 91 | Vacant 81. All values are ≥ 0.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>A. SECTION SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Required Count</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Filled Count</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Vacant</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Fill %</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>ELV / SCADA</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>67%</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>On Track</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>89</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>49%</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="n">
+        <v>172</v>
+      </c>
+      <c r="C12" s="13" t="n">
+        <v>91</v>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>81</v>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>53%</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>B. VACANT POSITIONS DETAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Designation</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Location / Area</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Vacant Count</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Required Count</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Filled Count</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Vacant</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Hiring Priority</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>ELV / SCADA</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Floor Technicians</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>PTB</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>ELV / SCADA</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Supervisior</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>PTB</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>ELV / SCADA</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Engineers</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>PTB</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>ELV / SCADA</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Supervisior</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Airside</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>MECHANICAL</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Sewerman &amp; Drainage</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>ALS QRT</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F9" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>ELECTRICAL</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>MRSS Operators (Sr Technician)</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>MRSS</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>ELECTRICAL</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Technicians (ELE -Ops)</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Admin building</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F11" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>ELECTRICAL</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Technicians (MST)</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Airside</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>MECHANICAL</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>HVAC Sr Technicians (chiller plant)</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Chiller plant</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F13" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>MECHANICAL</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Pump operator</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>CFR Satellite</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F14" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>MECHANICAL</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>STP helper</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>STP</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F15" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ELV / SCADA</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Sewage pump operator</t>
+          <t>Floor Technicians</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>ALS QRT</t>
+          <t>PTB</t>
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>6</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ELV / SCADA</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Helper Tech Associate Plu</t>
+          <t>Supervisior</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Admin building</t>
+          <t>PTB</t>
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>2</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ELV / SCADA</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Plumbing -Tech</t>
+          <t>Engineers</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Admin building</t>
+          <t>PTB</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>1</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ELV / SCADA</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Pump Operator</t>
+          <t>Supervisior</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>RO/firepump room</t>
+          <t>Airside</t>
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>1</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
@@ -4250,7 +4530,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Technician-mech</t>
+          <t>Sewerman &amp; Drainage</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -4259,9 +4539,15 @@
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
+        <v>6</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -4269,7 +4555,7 @@
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
@@ -4278,18 +4564,24 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Shift Engineers</t>
+          <t>MRSS Operators (Sr Technician)</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Overall ALS</t>
+          <t>MRSS</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" s="11" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H21" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -4297,16 +4589,16 @@
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ELECTRICAL</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Helper Tech Associate Mech.</t>
+          <t>Technicians (ELE -Ops)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -4315,9 +4607,15 @@
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F22" s="11" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -4325,27 +4623,33 @@
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ELECTRICAL</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Shift Engineers</t>
+          <t>Technicians (MST)</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>AIRSIDE &amp; Landside</t>
+          <t>Airside</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H23" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -4353,203 +4657,245 @@
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>High raise machine operators 21mt&amp; 18mt</t>
+          <t>HVAC Sr Technicians (chiller plant)</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>Chiller plant</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
+        <v>4</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>HSE &amp; Compliance Manager</t>
+          <t>Pump operator</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>CFR Satellite</t>
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
+        <v>4</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Materials Manager</t>
+          <t>STP helper</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>STP</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
+        <v>4</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Sr. Manager (Civil)</t>
+          <t>Sewage pump operator</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>ALS QRT</t>
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
+        <v>4</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Sr. Manager (Electrical)</t>
+          <t>Helper Tech Associate Plu</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>Admin building</t>
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
+        <v>3</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H28" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Sr. Manager (Mechanical)</t>
+          <t>Plumbing -Tech</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>Admin building</t>
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
+        <v>3</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>ELECTRICAL</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Shift Engineers</t>
+          <t>Pump Operator</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>PTB</t>
+          <t>RO/firepump room</t>
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>3</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H30" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
@@ -4558,54 +4904,66 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Asst Manager</t>
+          <t>Technician-mech</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>ALS QRT</t>
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>3</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ELECTRICAL</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>STP incharge</t>
+          <t>Shift Engineers</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>WTP</t>
+          <t>Overall ALS</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>2</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
@@ -4614,26 +4972,32 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>STP operator</t>
+          <t>Helper Tech Associate Mech.</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>STP</t>
+          <t>Admin building</t>
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>2</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
@@ -4642,315 +5006,681 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Safety Officer</t>
+          <t>Shift Engineers</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>ALS QRT</t>
+          <t>AIRSIDE &amp; Landside</t>
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>2</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>TRANSPORT</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Shift Engineers</t>
+          <t>High raise machine operators 21mt&amp; 18mt</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>PTB</t>
+          <t>TRANSPORT</t>
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>2</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>WTP Helper</t>
+          <t>HSE &amp; Compliance Manager</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>WTP</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="E36" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="F36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>WTP technician</t>
+          <t>Materials Manager</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>WTP</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="E37" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="F37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Associate mgr/JM</t>
+          <t>Sr. Manager (Civil)</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="E38" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F38" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="F38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Mechanical Helper</t>
+          <t>Sr. Manager (Electrical)</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="E39" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F39" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="F39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Paint machine operator</t>
+          <t>Sr. Manager (Mechanical)</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="E40" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F40" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="F40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Shift Engineers</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>PTB</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Asst Manager</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>STP incharge</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>WTP</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>STP operator</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>STP</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Safety Officer</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>ALS QRT</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Shift Engineers</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>PTB</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>WTP Helper</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>WTP</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>WTP technician</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>WTP</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Associate mgr/JM</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Mechanical Helper</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Paint machine operator</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" s="8" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>TRANSPORT</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>Tyre Technician</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D52" s="5" t="inlineStr">
         <is>
           <t>TRANSPORT</t>
         </is>
       </c>
-      <c r="E41" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="8" t="inlineStr">
+      <c r="E52" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" s="8" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="16" t="n"/>
-      <c r="B42" s="15" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="15" t="n"/>
+      <c r="B53" s="15" t="inlineStr">
         <is>
           <t>TOTAL VACANT</t>
         </is>
       </c>
-      <c r="C42" s="16" t="n"/>
-      <c r="D42" s="16" t="n"/>
-      <c r="E42" s="15" t="n">
+      <c r="C53" s="15" t="n"/>
+      <c r="D53" s="15" t="n"/>
+      <c r="E53" s="15" t="n">
         <v>81</v>
       </c>
-      <c r="F42" s="16" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>Section-wise vacant summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Vacant</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="21" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="B46" s="22" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="21" t="inlineStr">
-        <is>
-          <t>CIVIL</t>
-        </is>
-      </c>
-      <c r="B47" s="23" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="21" t="inlineStr">
-        <is>
-          <t>ELV / SCADA</t>
-        </is>
-      </c>
-      <c r="B48" s="24" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="21" t="inlineStr">
-        <is>
-          <t>ELECTRICAL</t>
-        </is>
-      </c>
-      <c r="B49" s="22" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="21" t="inlineStr">
-        <is>
-          <t>MECHANICAL</t>
-        </is>
-      </c>
-      <c r="B50" s="22" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="21" t="inlineStr">
-        <is>
-          <t>TRANSPORT</t>
-        </is>
-      </c>
-      <c r="B51" s="22" t="n">
-        <v>6</v>
-      </c>
-    </row>
+      <c r="F53" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="15" t="n">
+        <v>81</v>
+      </c>
+      <c r="H53" s="15" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>C. CROSS-CHECK</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="41" t="inlineStr">
+        <is>
+          <t>Deployment172: 91 named + 81 empty-name = 172. Summary172 Transport vacant corrected 7→6; TOTAL vacant corrected 82→81. Required / Filled / Vacant are all ≥ 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57"/>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A56:H57"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4979,6 +5709,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -5203,6 +5934,7 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -5363,6 +6095,8 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
@@ -5376,6 +6110,8 @@
           <t>• Full Plan: 281 required | 159 available (141 deployed + 18 will join) | Gap 122 (43%).</t>
         </is>
       </c>
+      <c r="B29" s="42" t="n"/>
+      <c r="C29" s="43" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="32" t="inlineStr">
@@ -5383,6 +6119,8 @@
           <t>• Phase-1 Immediate: 172 required | 91 named on roster (53%) | 81 vacant (47%).</t>
         </is>
       </c>
+      <c r="B30" s="42" t="n"/>
+      <c r="C30" s="43" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="32" t="inlineStr">
@@ -5390,6 +6128,8 @@
           <t>• Deferred beyond Phase-1: 109 positions.</t>
         </is>
       </c>
+      <c r="B31" s="42" t="n"/>
+      <c r="C31" s="43" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="32" t="inlineStr">
@@ -5397,6 +6137,8 @@
           <t>• Critical open: ELV/SCADA 10/10 vacant; Admin leadership 5 open; Mechanical largest vacant volume.</t>
         </is>
       </c>
+      <c r="B32" s="42" t="n"/>
+      <c r="C32" s="43" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="32" t="inlineStr">
@@ -5404,6 +6146,8 @@
           <t>• Top 281 gaps: Runway Team 13, HVAC Tech 10, Civil Helper 8, Pump Operator 8, Elec Shift Eng 7.</t>
         </is>
       </c>
+      <c r="B33" s="42" t="n"/>
+      <c r="C33" s="43" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -5424,7 +6168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -5438,6 +6182,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -5505,6 +6250,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -5632,6 +6378,8 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="33" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update Phase-1 vacancies detail with Required, Filled, Vacant Count
Sheet 4 designation detail now lists all Phase-1 slots by section/designation/location with Required Count, Filled Count, Vacant Count, and Hiring Priority. Section summary unchanged; totals remain 172 / 91 / 81.

Co-authored-by: Srikar Bokka <Srikar6266@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Phase1_172_vs_281_Manpower_Analysis_Report.xlsx
+++ b/Phase1_172_vs_281_Manpower_Analysis_Report.xlsx
@@ -113,7 +113,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -228,11 +228,12 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -323,6 +324,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -877,7 +883,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1107,7 +1112,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -1141,7 +1145,6 @@
       <c r="F20" s="39" t="n"/>
       <c r="G20" s="40" t="n"/>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
@@ -1363,7 +1366,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
@@ -1946,7 +1948,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -1963,7 +1964,6 @@
     </row>
     <row r="18"/>
     <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -4086,16 +4086,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -4335,11 +4335,21 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>B. VACANT POSITIONS DETAIL</t>
-        </is>
-      </c>
+      <c r="A14" s="44" t="inlineStr">
+        <is>
+          <t>B. DESIGNATION DETAIL — Required Count / Filled Count / Vacant Count</t>
+        </is>
+      </c>
+      <c r="B14" s="45" t="n"/>
+      <c r="C14" s="45" t="n"/>
+      <c r="D14" s="45" t="n"/>
+      <c r="E14" s="45" t="n"/>
+      <c r="F14" s="45" t="n"/>
+      <c r="G14" s="45" t="n"/>
+      <c r="H14" s="45" t="n"/>
+      <c r="I14" s="45" t="n"/>
+      <c r="J14" s="45" t="n"/>
+      <c r="K14" s="45" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -4374,7 +4384,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Vacant</t>
+          <t>Vacant Count</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -4382,6 +4392,9 @@
           <t>Hiring Priority</t>
         </is>
       </c>
+      <c r="I15" s="45" t="n"/>
+      <c r="J15" s="45" t="n"/>
+      <c r="K15" s="45" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
@@ -4408,7 +4421,7 @@
       <c r="F16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="7" t="n">
+      <c r="G16" s="10" t="n">
         <v>6</v>
       </c>
       <c r="H16" s="10" t="inlineStr">
@@ -4416,6 +4429,9 @@
           <t>CRITICAL</t>
         </is>
       </c>
+      <c r="I16" s="45" t="n"/>
+      <c r="J16" s="45" t="n"/>
+      <c r="K16" s="45" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
@@ -4442,7 +4458,7 @@
       <c r="F17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="7" t="n">
+      <c r="G17" s="10" t="n">
         <v>2</v>
       </c>
       <c r="H17" s="10" t="inlineStr">
@@ -4450,6 +4466,9 @@
           <t>CRITICAL</t>
         </is>
       </c>
+      <c r="I17" s="45" t="n"/>
+      <c r="J17" s="45" t="n"/>
+      <c r="K17" s="45" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
@@ -4476,7 +4495,7 @@
       <c r="F18" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="7" t="n">
+      <c r="G18" s="10" t="n">
         <v>1</v>
       </c>
       <c r="H18" s="10" t="inlineStr">
@@ -4484,6 +4503,9 @@
           <t>CRITICAL</t>
         </is>
       </c>
+      <c r="I18" s="45" t="n"/>
+      <c r="J18" s="45" t="n"/>
+      <c r="K18" s="45" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
@@ -4510,7 +4532,7 @@
       <c r="F19" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="7" t="n">
+      <c r="G19" s="10" t="n">
         <v>1</v>
       </c>
       <c r="H19" s="10" t="inlineStr">
@@ -4518,6 +4540,9 @@
           <t>CRITICAL</t>
         </is>
       </c>
+      <c r="I19" s="45" t="n"/>
+      <c r="J19" s="45" t="n"/>
+      <c r="K19" s="45" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
@@ -4525,33 +4550,36 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Sewerman &amp; Drainage</t>
+          <t>HSE &amp; Compliance Manager</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>ALS QRT</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F20" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
+      <c r="G20" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="I20" s="45" t="n"/>
+      <c r="J20" s="45" t="n"/>
+      <c r="K20" s="45" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
@@ -4559,33 +4587,36 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>ELECTRICAL</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>MRSS Operators (Sr Technician)</t>
+          <t>Materials Manager</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>MRSS</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H21" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
+      <c r="G21" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="I21" s="45" t="n"/>
+      <c r="J21" s="45" t="n"/>
+      <c r="K21" s="45" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
@@ -4593,33 +4624,36 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>ELECTRICAL</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Technicians (ELE -Ops)</t>
+          <t>Sr. Manager (Civil)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Admin building</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H22" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
+      <c r="G22" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="I22" s="45" t="n"/>
+      <c r="J22" s="45" t="n"/>
+      <c r="K22" s="45" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
@@ -4627,33 +4661,36 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>ELECTRICAL</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Technicians (MST)</t>
+          <t>Sr. Manager (Electrical)</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Airside</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F23" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G23" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H23" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
+      <c r="G23" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="I23" s="45" t="n"/>
+      <c r="J23" s="45" t="n"/>
+      <c r="K23" s="45" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
@@ -4661,33 +4698,36 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>HVAC Sr Technicians (chiller plant)</t>
+          <t>Sr. Manager (Mechanical)</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Chiller plant</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G24" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H24" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
+      <c r="G24" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="I24" s="45" t="n"/>
+      <c r="J24" s="45" t="n"/>
+      <c r="K24" s="45" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
@@ -4695,17 +4735,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ELECTRICAL</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Pump operator</t>
+          <t>MRSS Operators (Sr Technician)</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>CFR Satellite</t>
+          <t>MRSS</t>
         </is>
       </c>
       <c r="E25" s="6" t="n">
@@ -4714,7 +4754,7 @@
       <c r="F25" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="7" t="n">
+      <c r="G25" s="10" t="n">
         <v>4</v>
       </c>
       <c r="H25" s="11" t="inlineStr">
@@ -4722,6 +4762,9 @@
           <t>HIGH</t>
         </is>
       </c>
+      <c r="I25" s="45" t="n"/>
+      <c r="J25" s="45" t="n"/>
+      <c r="K25" s="45" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
@@ -4729,17 +4772,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ELECTRICAL</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>STP helper</t>
+          <t>Technicians (ELE -Ops)</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>STP</t>
+          <t>Admin building</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
@@ -4748,7 +4791,7 @@
       <c r="F26" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G26" s="7" t="n">
+      <c r="G26" s="10" t="n">
         <v>4</v>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -4756,6 +4799,9 @@
           <t>HIGH</t>
         </is>
       </c>
+      <c r="I26" s="45" t="n"/>
+      <c r="J26" s="45" t="n"/>
+      <c r="K26" s="45" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
@@ -4763,17 +4809,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ELECTRICAL</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Sewage pump operator</t>
+          <t>Technicians (MST)</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>ALS QRT</t>
+          <t>Airside</t>
         </is>
       </c>
       <c r="E27" s="6" t="n">
@@ -4782,7 +4828,7 @@
       <c r="F27" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="7" t="n">
+      <c r="G27" s="10" t="n">
         <v>4</v>
       </c>
       <c r="H27" s="11" t="inlineStr">
@@ -4790,6 +4836,9 @@
           <t>HIGH</t>
         </is>
       </c>
+      <c r="I27" s="45" t="n"/>
+      <c r="J27" s="45" t="n"/>
+      <c r="K27" s="45" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
@@ -4797,33 +4846,36 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ELECTRICAL</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Helper Tech Associate Plu</t>
+          <t>Shift Engineers</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Admin building</t>
+          <t>Overall ALS</t>
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F28" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="7" t="n">
-        <v>3</v>
+      <c r="G28" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
+      <c r="I28" s="45" t="n"/>
+      <c r="J28" s="45" t="n"/>
+      <c r="K28" s="45" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
@@ -4831,33 +4883,36 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>ELECTRICAL</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Plumbing -Tech</t>
+          <t>Shift Engineers</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Admin building</t>
+          <t>PTB</t>
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>HIGH</t>
-        </is>
-      </c>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I29" s="45" t="n"/>
+      <c r="J29" s="45" t="n"/>
+      <c r="K29" s="45" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
@@ -4870,28 +4925,31 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Pump Operator</t>
+          <t>Sewerman &amp; Drainage</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>RO/firepump room</t>
+          <t>ALS QRT</t>
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F30" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G30" s="7" t="n">
-        <v>3</v>
+      <c r="G30" s="10" t="n">
+        <v>6</v>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
+      <c r="I30" s="45" t="n"/>
+      <c r="J30" s="45" t="n"/>
+      <c r="K30" s="45" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
@@ -4904,28 +4962,31 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Technician-mech</t>
+          <t>HVAC Sr Technicians (chiller plant)</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>ALS QRT</t>
+          <t>Chiller plant</t>
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F31" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="7" t="n">
-        <v>3</v>
+      <c r="G31" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
+      <c r="I31" s="45" t="n"/>
+      <c r="J31" s="45" t="n"/>
+      <c r="K31" s="45" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
@@ -4933,33 +4994,36 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>ELECTRICAL</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Shift Engineers</t>
+          <t>Pump operator</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Overall ALS</t>
+          <t>CFR Satellite</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F32" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G32" s="7" t="n">
-        <v>2</v>
+      <c r="G32" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
+      <c r="I32" s="45" t="n"/>
+      <c r="J32" s="45" t="n"/>
+      <c r="K32" s="45" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
@@ -4972,28 +5036,31 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Helper Tech Associate Mech.</t>
+          <t>STP helper</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Admin building</t>
+          <t>STP</t>
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F33" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G33" s="7" t="n">
-        <v>2</v>
+      <c r="G33" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
+      <c r="I33" s="45" t="n"/>
+      <c r="J33" s="45" t="n"/>
+      <c r="K33" s="45" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
@@ -5006,28 +5073,31 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Shift Engineers</t>
+          <t>Sewage pump operator</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>AIRSIDE &amp; Landside</t>
+          <t>ALS QRT</t>
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F34" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G34" s="7" t="n">
-        <v>2</v>
+      <c r="G34" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
+      <c r="I34" s="45" t="n"/>
+      <c r="J34" s="45" t="n"/>
+      <c r="K34" s="45" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
@@ -5035,33 +5105,36 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>High raise machine operators 21mt&amp; 18mt</t>
+          <t>Helper Tech Associate Plu</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>Admin building</t>
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F35" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G35" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H35" s="7" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
+      <c r="G35" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H35" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="I35" s="45" t="n"/>
+      <c r="J35" s="45" t="n"/>
+      <c r="K35" s="45" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
@@ -5069,33 +5142,36 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>HSE &amp; Compliance Manager</t>
+          <t>Plumbing -Tech</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>Admin building</t>
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F36" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G36" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H36" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
+      <c r="G36" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H36" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="I36" s="45" t="n"/>
+      <c r="J36" s="45" t="n"/>
+      <c r="K36" s="45" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
@@ -5103,33 +5179,36 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Materials Manager</t>
+          <t>Pump Operator</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>RO/firepump room</t>
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F37" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G37" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H37" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
+      <c r="G37" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H37" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="I37" s="45" t="n"/>
+      <c r="J37" s="45" t="n"/>
+      <c r="K37" s="45" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
@@ -5137,33 +5216,36 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Sr. Manager (Civil)</t>
+          <t>Technician-mech</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>ALS QRT</t>
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H38" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="H38" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="I38" s="45" t="n"/>
+      <c r="J38" s="45" t="n"/>
+      <c r="K38" s="45" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
@@ -5171,33 +5253,36 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Sr. Manager (Electrical)</t>
+          <t>Helper Tech Associate Mech.</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>Admin building</t>
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F39" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G39" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H39" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
+      <c r="G39" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="I39" s="45" t="n"/>
+      <c r="J39" s="45" t="n"/>
+      <c r="K39" s="45" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
@@ -5205,33 +5290,36 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Sr. Manager (Mechanical)</t>
+          <t>Shift Engineers</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>AIRSIDE &amp; Landside</t>
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F40" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G40" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H40" s="10" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
+      <c r="G40" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="I40" s="45" t="n"/>
+      <c r="J40" s="45" t="n"/>
+      <c r="K40" s="45" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
@@ -5239,17 +5327,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>ELECTRICAL</t>
+          <t>MECHANICAL</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Shift Engineers</t>
+          <t>Asst Manager</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>PTB</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="E41" s="6" t="n">
@@ -5258,14 +5346,17 @@
       <c r="F41" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G41" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H41" s="8" t="inlineStr">
+      <c r="G41" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" s="11" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
+      <c r="I41" s="45" t="n"/>
+      <c r="J41" s="45" t="n"/>
+      <c r="K41" s="45" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
@@ -5278,12 +5369,12 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Asst Manager</t>
+          <t>STP incharge</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>WTP</t>
         </is>
       </c>
       <c r="E42" s="6" t="n">
@@ -5292,14 +5383,17 @@
       <c r="F42" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G42" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H42" s="8" t="inlineStr">
+      <c r="G42" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" s="11" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
+      <c r="I42" s="45" t="n"/>
+      <c r="J42" s="45" t="n"/>
+      <c r="K42" s="45" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
@@ -5312,28 +5406,31 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>STP incharge</t>
+          <t>STP operator</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>WTP</t>
+          <t>STP</t>
         </is>
       </c>
       <c r="E43" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G43" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H43" s="8" t="inlineStr">
+      <c r="H43" s="11" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
+      <c r="I43" s="45" t="n"/>
+      <c r="J43" s="45" t="n"/>
+      <c r="K43" s="45" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n">
@@ -5346,12 +5443,12 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>STP operator</t>
+          <t>Safety Officer</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>STP</t>
+          <t>ALS QRT</t>
         </is>
       </c>
       <c r="E44" s="6" t="n">
@@ -5360,14 +5457,17 @@
       <c r="F44" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G44" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H44" s="8" t="inlineStr">
+      <c r="G44" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="11" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
+      <c r="I44" s="45" t="n"/>
+      <c r="J44" s="45" t="n"/>
+      <c r="K44" s="45" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
@@ -5380,12 +5480,12 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Safety Officer</t>
+          <t>Shift Engineers</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>ALS QRT</t>
+          <t>PTB</t>
         </is>
       </c>
       <c r="E45" s="6" t="n">
@@ -5394,14 +5494,17 @@
       <c r="F45" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G45" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H45" s="8" t="inlineStr">
+      <c r="G45" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" s="11" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
+      <c r="I45" s="45" t="n"/>
+      <c r="J45" s="45" t="n"/>
+      <c r="K45" s="45" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
@@ -5414,28 +5517,31 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Shift Engineers</t>
+          <t>WTP Helper</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>PTB</t>
+          <t>WTP</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F46" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G46" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H46" s="8" t="inlineStr">
+      <c r="H46" s="11" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
+      <c r="I46" s="45" t="n"/>
+      <c r="J46" s="45" t="n"/>
+      <c r="K46" s="45" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
@@ -5448,7 +5554,7 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>WTP Helper</t>
+          <t>WTP technician</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
@@ -5457,19 +5563,22 @@
         </is>
       </c>
       <c r="E47" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F47" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G47" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H47" s="8" t="inlineStr">
+      <c r="H47" s="11" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
+      <c r="I47" s="45" t="n"/>
+      <c r="J47" s="45" t="n"/>
+      <c r="K47" s="45" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n">
@@ -5477,33 +5586,36 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>MECHANICAL</t>
+          <t>TRANSPORT</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>WTP technician</t>
+          <t>High raise machine operators 21mt&amp; 18mt</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>WTP</t>
+          <t>TRANSPORT</t>
         </is>
       </c>
       <c r="E48" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F48" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G48" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H48" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
+      <c r="G48" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I48" s="45" t="n"/>
+      <c r="J48" s="45" t="n"/>
+      <c r="K48" s="45" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n">
@@ -5530,14 +5642,17 @@
       <c r="F49" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G49" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H49" s="8" t="inlineStr">
+      <c r="G49" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" s="11" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
+      <c r="I49" s="45" t="n"/>
+      <c r="J49" s="45" t="n"/>
+      <c r="K49" s="45" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n">
@@ -5564,14 +5679,17 @@
       <c r="F50" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G50" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H50" s="8" t="inlineStr">
+      <c r="G50" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" s="11" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
+      <c r="I50" s="45" t="n"/>
+      <c r="J50" s="45" t="n"/>
+      <c r="K50" s="45" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n">
@@ -5598,14 +5716,17 @@
       <c r="F51" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G51" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H51" s="8" t="inlineStr">
+      <c r="G51" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" s="11" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
+      <c r="I51" s="45" t="n"/>
+      <c r="J51" s="45" t="n"/>
+      <c r="K51" s="45" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
@@ -5632,53 +5753,1681 @@
       <c r="F52" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G52" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H52" s="8" t="inlineStr">
+      <c r="G52" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" s="11" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
+      <c r="I52" s="45" t="n"/>
+      <c r="J52" s="45" t="n"/>
+      <c r="K52" s="45" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="15" t="n"/>
-      <c r="B53" s="15" t="inlineStr">
-        <is>
-          <t>TOTAL VACANT</t>
-        </is>
-      </c>
-      <c r="C53" s="15" t="n"/>
-      <c r="D53" s="15" t="n"/>
-      <c r="E53" s="15" t="n">
+      <c r="A53" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>HR Manager</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I53" s="45" t="n"/>
+      <c r="J53" s="45" t="n"/>
+      <c r="K53" s="45" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>MIS Executive</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I54" s="45" t="n"/>
+      <c r="J54" s="45" t="n"/>
+      <c r="K54" s="45" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Site Head (GM)</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I55" s="45" t="n"/>
+      <c r="J55" s="45" t="n"/>
+      <c r="K55" s="45" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Asst Manager</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I56" s="45" t="n"/>
+      <c r="J56" s="45" t="n"/>
+      <c r="K56" s="45" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Floor Technicians</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F57" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G57" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I57" s="45" t="n"/>
+      <c r="J57" s="45" t="n"/>
+      <c r="K57" s="45" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>High Mast Operator (Technicians)</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>High Mast</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I58" s="45" t="n"/>
+      <c r="J58" s="45" t="n"/>
+      <c r="K58" s="45" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>MRSS Operators (Technician)</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>MRSS</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I59" s="45" t="n"/>
+      <c r="J59" s="45" t="n"/>
+      <c r="K59" s="45" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>MRSS Operators (Technician)</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F60" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G60" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I60" s="45" t="n"/>
+      <c r="J60" s="45" t="n"/>
+      <c r="K60" s="45" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Ops Technicians (ELE -Ops)</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>AGL-EAST</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I61" s="45" t="n"/>
+      <c r="J61" s="45" t="n"/>
+      <c r="K61" s="45" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Ops Technicians (ELE -Ops)</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>AGL-WEST</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F62" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G62" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Sr Technicians</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>MRSS</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F63" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G63" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Substation Operators</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>AGL-EAST</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F64" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G64" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Substation Operators</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G65" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Substation Operators</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Technicians</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Landside</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F67" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G67" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Fitter Mechanical</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>HVAC Floor Technicians</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>HVAC Floor Technicians</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>ATC</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>HVAC Floor Technicians</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>HVAC Floor Technicians</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>PTB</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F72" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G72" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>HVAC Floor Technicians</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F73" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G73" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Helper (Tech-Ass-Mec) chiller plant</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F74" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G74" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Helper Tech Associate Mech.</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>ADMIN/MRSS</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F75" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="n">
+        <v>61</v>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Helper Tech Associate Mech.</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>ALS QRT</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F76" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G76" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Helper Tech Associate Mech.</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F77" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G77" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Helper Utility building</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Airside</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Plumbing Technican</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>ATC Pump House</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F79" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G79" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="n">
+        <v>65</v>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Plumbing Technican</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F80" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G80" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Plumbing Technican</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>CFR Pump House</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F81" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G81" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="n">
+        <v>67</v>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Plumbing Technican</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>East Side</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>Plumbing Technican</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>PTB</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F83" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="n">
+        <v>69</v>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Plumbing Technican</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>West Side</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F84" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G84" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Pump Operator</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F85" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Shift Engineers</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="E86" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F86" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Technician-mech</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>ATC</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Technician-mech</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>PTB</t>
+        </is>
+      </c>
+      <c r="E88" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F88" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G88" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="n">
+        <v>74</v>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>MECHANICAL</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Technician-mech</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="E89" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G89" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Motor Electrician</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="E90" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G90" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Motor Technician</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F91" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="n">
+        <v>77</v>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Road sweeper operator</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="E92" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F92" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G92" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>Carpenter</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>PTB</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F93" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Civil Fitter</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>PTB</t>
+        </is>
+      </c>
+      <c r="E94" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F94" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G94" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>Civil Helper</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>Airside</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F95" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G95" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="n">
         <v>81</v>
       </c>
-      <c r="F53" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="15" t="n">
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>Engr</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>PTB</t>
+        </is>
+      </c>
+      <c r="E96" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F96" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G96" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Supervisor Civil</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>ALS</t>
+        </is>
+      </c>
+      <c r="E97" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F97" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G97" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>Supervisor Civil</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>PTB</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G98" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Welder</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>PTB</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F99" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G99" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="12" t="n"/>
+      <c r="B100" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C100" s="12" t="n"/>
+      <c r="D100" s="12" t="n"/>
+      <c r="E100" s="13" t="n">
+        <v>172</v>
+      </c>
+      <c r="F100" s="13" t="n">
+        <v>91</v>
+      </c>
+      <c r="G100" s="13" t="n">
         <v>81</v>
       </c>
-      <c r="H53" s="15" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="H100" s="12" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
         <is>
           <t>C. CROSS-CHECK</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="41" t="inlineStr">
-        <is>
-          <t>Deployment172: 91 named + 81 empty-name = 172. Summary172 Transport vacant corrected 7→6; TOTAL vacant corrected 82→81. Required / Filled / Vacant are all ≥ 0.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57"/>
+    <row r="103">
+      <c r="A103" s="46" t="inlineStr">
+        <is>
+          <t>Deployment172: Required 172 | Filled 91 | Vacant 81. Vacant Count = Required Count − Filled Count (always ≥ 0). Section A unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A56:H57"/>
+    <mergeCell ref="A103:H104"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -5709,7 +7458,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -5934,7 +7682,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -6095,8 +7842,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
@@ -6168,7 +7913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -6182,7 +7927,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -6250,7 +7994,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -6378,8 +8121,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="33" t="inlineStr">
         <is>

</xml_diff>